<commit_message>
revisi admin customer tahap 1
</commit_message>
<xml_diff>
--- a/DAFTAR REVISI.xlsx
+++ b/DAFTAR REVISI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\V1 Flutter\chupatu_mobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51AA6E3D-A488-467B-B288-6391AD8B30E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DD449EA-8828-4EAE-8B3A-33F66B219609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{408ADA03-67D4-4BA9-9259-15D9795C01CA}"/>
   </bookViews>
@@ -1109,7 +1109,9 @@
       <c r="G19" s="6"/>
     </row>
     <row r="20" spans="1:7" ht="48.6" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="4"/>
+      <c r="A20" s="4">
+        <v>16</v>
+      </c>
       <c r="B20" s="5" t="s">
         <v>33</v>
       </c>

</xml_diff>

<commit_message>
revisi admin customer tahap 1.1
</commit_message>
<xml_diff>
--- a/DAFTAR REVISI.xlsx
+++ b/DAFTAR REVISI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\V1 Flutter\chupatu_mobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DD449EA-8828-4EAE-8B3A-33F66B219609}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{946CF19B-8C45-4B48-848B-C1E08821EBC8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{408ADA03-67D4-4BA9-9259-15D9795C01CA}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
   <si>
     <t>REVISI CHUPATU MOBILE</t>
   </si>
@@ -90,9 +90,6 @@
     <t>CUSTOMER</t>
   </si>
   <si>
-    <t>FITUR FORGOT PASSWORD BELUM JADI</t>
-  </si>
-  <si>
     <t>FITUR CHECK EMAIL ASLI DI SIGN UP BELUM ADA</t>
   </si>
   <si>
@@ -108,9 +105,6 @@
     <t>FITUR CEK KONDISI AI DI BAGIAN + HOME PAGE ITU BELUM ADA, BAGUS NYA ADA LOGIC DEEP LEARNING DISITU JADI BISA NGEBACA INI JENIS SEPATU APA, KODISINYA GMN JADI DIA REKOMENIN PESANAN YANG COCOK GMN, TRUS NGASIH REKOMEN PERAWATANNYA GMN.</t>
   </si>
   <si>
-    <t>FITUR TEMA DITAMBAH LAGI : NEUMORPHISM, GLASSMORPHISM, IMMERSIVE 3D, RETRO,DARK MODERN</t>
-  </si>
-  <si>
     <t>FITUR FITUR DI PENGATURAN AKUN JADIIN SEMUA YA BABI</t>
   </si>
   <si>
@@ -129,20 +123,47 @@
     <t>HARDCORE</t>
   </si>
   <si>
-    <t>fitur gudang itu nanti adakan untuk input harga beli barang, terus juga bisa edit harga yang sudah tercatat saat menambahkan barang nya</t>
-  </si>
-  <si>
     <t>NOTE</t>
   </si>
   <si>
     <t>DI FITUR KASIR JIKA ADMIN TAMBAH LAYANAN BARU TUH GA TAMPIL DI BAGIAN KASIR INI</t>
+  </si>
+  <si>
+    <t>FITUR FORGOT PASSWORD BELUM JADI (MASUK KE SPAM EMAILNYA)</t>
+  </si>
+  <si>
+    <t>FITUR TEMA DITAMBAH LAGI : NEUMORPHISM, GLASSMORPHISM, IMMERSIVE 3D, RETRO,DARK MODERN,DI MENU NOTIF ITU KADANG TEMA NYA GA JALAN</t>
+  </si>
+  <si>
+    <t>FITUR GUDANG ITU NANTI ADAKAN UNTUK INPUT HARGA BELI BARANG, TERUS JUGA BISA EDIT HARGA YANG SUDAH TERCATAT SAAT MENAMBAHKAN BARANG NYA. JADI NANTI DI LAPORAN KELUAR ITU BISA TRACK HARGA</t>
+  </si>
+  <si>
+    <t>TEMA GLASS DI ADMIN TERLALU BERAT DI MOBILE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MENU ORDER IKONNYA ILANG </t>
+  </si>
+  <si>
+    <t>FITUR DI DATA PELANGGAN KURANG UNTUK FILTER BERDASARKAN JUMLAH PESANAN DAN HARGA TERBESAR</t>
+  </si>
+  <si>
+    <t>DI MENU ORDER, DAFTAR PESANANNYA FILTERNYA KURANG LENGKAP</t>
+  </si>
+  <si>
+    <t>TOMBOL NOTIF ITU IKONNYA ADA MERAHNYA SAAT ADA NOTIF TERBARU AJA DAN BISA GOYANG GOYANG KETIKA ADA NOTIF BARU YANG BELUM DIBUKA</t>
+  </si>
+  <si>
+    <t>LAYANAN CUSTOM ITU MAKSUDNYA DIA BISA PILIH BEBERAPA SEKALIGUS, NANTI DIBUAT LEBIH LENGKAP</t>
+  </si>
+  <si>
+    <t>FITUR CHUPATU PRO INI, NANTI APA MASUK DI LAPORAN PEMASUKAN ATAU GMN YA?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -187,6 +208,31 @@
       <name val="Arial Black"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial Black"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -214,7 +260,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -225,6 +271,59 @@
     <border>
       <left/>
       <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
       <top style="thin">
         <color theme="4" tint="0.39997558519241921"/>
       </top>
@@ -237,7 +336,7 @@
       <left style="thick">
         <color indexed="64"/>
       </left>
-      <right style="thick">
+      <right style="double">
         <color indexed="64"/>
       </right>
       <top style="thick">
@@ -250,7 +349,7 @@
       <left style="thick">
         <color indexed="64"/>
       </left>
-      <right style="thick">
+      <right style="double">
         <color indexed="64"/>
       </right>
       <top/>
@@ -261,9 +360,40 @@
       <left style="thick">
         <color indexed="64"/>
       </left>
-      <right style="thick">
+      <right style="double">
         <color indexed="64"/>
       </right>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color indexed="64"/>
+      </left>
+      <right/>
       <top/>
       <bottom style="thick">
         <color indexed="64"/>
@@ -274,7 +404,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -292,28 +422,73 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -321,6 +496,25 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -333,7 +527,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -348,20 +542,6 @@
         <scheme val="minor"/>
       </font>
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -402,7 +582,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -473,26 +653,26 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{17F41CE2-7A14-4B5F-8E68-95745F812320}" name="Table4" displayName="Table4" ref="A4:C20" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="A4:C20" xr:uid="{17F41CE2-7A14-4B5F-8E68-95745F812320}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{17F41CE2-7A14-4B5F-8E68-95745F812320}" name="Table4" displayName="Table4" ref="B4:D24" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="B4:D24" xr:uid="{17F41CE2-7A14-4B5F-8E68-95745F812320}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{42737F92-8B24-49D4-BAA2-9D264BB857C1}" name="NO" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{C7960063-BCB1-499F-8687-98DFBC7C5CFF}" name="ADMIN" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{3FCE4E8C-F710-47E1-933B-750F7465C90D}" name="PROGRES" dataDxfId="5"/>
+    <tableColumn id="5" xr3:uid="{B811EBC1-E8D7-43F4-AD43-47F971627D50}" name="NO" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{C7960063-BCB1-499F-8687-98DFBC7C5CFF}" name="ADMIN" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{3FCE4E8C-F710-47E1-933B-750F7465C90D}" name="PROGRES" dataDxfId="1"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D65A9FC3-111E-4033-88B4-1E149CEA158A}" name="Table5" displayName="Table5" ref="E4:G14" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
-  <autoFilter ref="E4:G14" xr:uid="{D65A9FC3-111E-4033-88B4-1E149CEA158A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D65A9FC3-111E-4033-88B4-1E149CEA158A}" name="Table5" displayName="Table5" ref="F4:H17" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
+  <autoFilter ref="F4:H17" xr:uid="{D65A9FC3-111E-4033-88B4-1E149CEA158A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{BA4067DE-A9E6-4A79-8183-BBDC9DCB5B98}" name="NO" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{5BEFE63E-C8A9-4CB7-B801-BC4E48F2A3CF}" name="CUSTOMER" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{F876FA39-0709-43F6-9198-5F2408DAB962}" name="PROGRES" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{BA4067DE-A9E6-4A79-8183-BBDC9DCB5B98}" name="NO" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{5BEFE63E-C8A9-4CB7-B801-BC4E48F2A3CF}" name="CUSTOMER" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{F876FA39-0709-43F6-9198-5F2408DAB962}" name="PROGRES" dataDxfId="5"/>
   </tableColumns>
-  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -793,333 +973,516 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01AD129F-D61F-4BD9-AB11-BBB76F78B373}">
-  <dimension ref="A2:G20"/>
+  <dimension ref="B2:J37"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.21875" customWidth="1"/>
-    <col min="2" max="2" width="90.77734375" customWidth="1"/>
-    <col min="3" max="3" width="11.77734375" customWidth="1"/>
-    <col min="4" max="4" width="8.44140625" customWidth="1"/>
-    <col min="5" max="5" width="9.21875" customWidth="1"/>
-    <col min="6" max="6" width="90.77734375" customWidth="1"/>
-    <col min="7" max="7" width="11.77734375" customWidth="1"/>
+    <col min="2" max="2" width="9.21875" customWidth="1"/>
+    <col min="3" max="3" width="90.77734375" customWidth="1"/>
+    <col min="4" max="4" width="11.77734375" customWidth="1"/>
+    <col min="5" max="5" width="8.44140625" customWidth="1"/>
+    <col min="6" max="6" width="9.21875" customWidth="1"/>
+    <col min="7" max="7" width="90.77734375" customWidth="1"/>
+    <col min="8" max="8" width="11.77734375" customWidth="1"/>
+    <col min="10" max="10" width="77.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:7" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="A2" s="9" t="s">
+    <row r="2" spans="2:10" ht="23.4" x14ac:dyDescent="0.45">
+      <c r="B2" s="9" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="9"/>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
       <c r="F2" s="9"/>
       <c r="G2" s="9"/>
-    </row>
-    <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="H2" s="9"/>
+    </row>
+    <row r="4" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" s="3"/>
+      <c r="F4" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="4">
+        <v>1</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" s="4">
+        <v>1</v>
+      </c>
+      <c r="E5" s="6"/>
+      <c r="F5" s="4">
+        <v>1</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="4">
+        <v>2</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="4">
+        <v>1</v>
+      </c>
+      <c r="E6" s="6"/>
+      <c r="F6" s="4">
+        <v>2</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="4">
+        <v>3</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="4">
+        <v>1</v>
+      </c>
+      <c r="E7" s="6"/>
+      <c r="F7" s="4">
+        <v>3</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" s="6">
+        <v>1</v>
+      </c>
+      <c r="J7" s="12"/>
+    </row>
+    <row r="8" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="4">
+        <v>4</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="4">
+        <v>1</v>
+      </c>
+      <c r="E8" s="6"/>
+      <c r="F8" s="4">
+        <v>4</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="H8" s="6"/>
+    </row>
+    <row r="9" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="4">
+        <v>5</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="4">
+        <v>1</v>
+      </c>
+      <c r="E9" s="6"/>
+      <c r="F9" s="4">
+        <v>5</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="6"/>
+    </row>
+    <row r="10" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="4">
+        <v>6</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="4">
+        <v>1</v>
+      </c>
+      <c r="E10" s="6"/>
+      <c r="F10" s="4">
+        <v>6</v>
+      </c>
+      <c r="G10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="H10" s="6"/>
+    </row>
+    <row r="11" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="4">
+        <v>7</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D11" s="4">
+        <v>1</v>
+      </c>
+      <c r="E11" s="6"/>
+      <c r="F11" s="4">
+        <v>7</v>
+      </c>
+      <c r="G11" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="4">
+        <v>8</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="4">
+        <v>1</v>
+      </c>
+      <c r="E12" s="6"/>
+      <c r="F12" s="4">
+        <v>8</v>
+      </c>
+      <c r="G12" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="H12" s="6"/>
+    </row>
+    <row r="13" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="4">
+        <v>9</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="4">
+        <v>1</v>
+      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="4">
+        <v>9</v>
+      </c>
+      <c r="G13" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="H13" s="6"/>
+    </row>
+    <row r="14" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="4">
+        <v>10</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" s="4">
+        <v>1</v>
+      </c>
+      <c r="E14" s="6"/>
+      <c r="F14" s="4">
+        <v>10</v>
+      </c>
+      <c r="G14" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="D4" s="3"/>
-      <c r="E4" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="H14" s="6"/>
+    </row>
+    <row r="15" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="4">
+        <v>11</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D15" s="8">
+        <v>1</v>
+      </c>
+      <c r="E15" s="6"/>
+      <c r="F15" s="4">
+        <v>11</v>
+      </c>
+      <c r="G15" s="5" t="str">
+        <f>UPPER("fitur kasih rating dan masuk ke halaman review our service dan di bagian bawah magic result yg rating")</f>
+        <v>FITUR KASIH RATING DAN MASUK KE HALAMAN REVIEW OUR SERVICE DAN DI BAGIAN BAWAH MAGIC RESULT YG RATING</v>
+      </c>
+      <c r="H15" s="6"/>
+    </row>
+    <row r="16" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="4">
+        <v>12</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" s="4">
+        <v>1</v>
+      </c>
+      <c r="E16" s="6"/>
+      <c r="F16" s="4">
+        <v>12</v>
+      </c>
+      <c r="G16" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H16" s="6"/>
+    </row>
+    <row r="17" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="4">
+        <v>13</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="4">
+        <v>1</v>
+      </c>
+      <c r="E17" s="6"/>
+      <c r="F17" s="4">
+        <v>13</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H17" s="6"/>
+    </row>
+    <row r="18" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="4">
+        <v>14</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D18" s="4">
+        <v>1</v>
+      </c>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="H18" s="6"/>
+    </row>
+    <row r="19" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="4">
+        <v>15</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D19" s="4">
+        <v>1</v>
+      </c>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="H19" s="6"/>
+    </row>
+    <row r="20" spans="2:8" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="4">
+        <v>16</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="D20" s="4"/>
+    </row>
+    <row r="21" spans="2:8" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="4">
         <v>17</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="4">
-        <v>1</v>
-      </c>
-      <c r="B5" s="5" t="s">
+      <c r="C21" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D21" s="4"/>
+    </row>
+    <row r="22" spans="2:8" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="4">
+        <v>18</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D22" s="4"/>
+    </row>
+    <row r="23" spans="2:8" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="4">
+        <v>19</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="D23" s="4"/>
+    </row>
+    <row r="24" spans="2:8" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="4">
+        <v>20</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="D24" s="4"/>
+    </row>
+    <row r="25" spans="2:8" ht="46.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
+    <row r="26" spans="2:8" ht="46.2" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D26" s="10"/>
+      <c r="E26" s="10"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="18"/>
+    </row>
+    <row r="27" spans="2:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="22">
+        <v>1</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>33</v>
+      </c>
+      <c r="D27" s="13"/>
+      <c r="E27" s="13"/>
+      <c r="F27" s="14"/>
+      <c r="G27" s="19"/>
+    </row>
+    <row r="28" spans="2:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="22">
         <v>2</v>
       </c>
-      <c r="C5" s="4">
-        <v>1</v>
-      </c>
-      <c r="D5" s="6"/>
-      <c r="E5" s="4">
-        <v>1</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="6"/>
-    </row>
-    <row r="6" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="4">
-        <v>2</v>
-      </c>
-      <c r="B6" s="5" t="s">
+      <c r="C28" s="17" t="str">
+        <f>UPPER("anti nama di profil belum sinkron dengan home untuk customer, ubah foto profil juga gabisa")</f>
+        <v>ANTI NAMA DI PROFIL BELUM SINKRON DENGAN HOME UNTUK CUSTOMER, UBAH FOTO PROFIL JUGA GABISA</v>
+      </c>
+      <c r="D28" s="13"/>
+      <c r="E28" s="13"/>
+      <c r="F28" s="14"/>
+      <c r="G28" s="19"/>
+    </row>
+    <row r="29" spans="2:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="22">
         <v>3</v>
       </c>
-      <c r="C6" s="4">
-        <v>1</v>
-      </c>
-      <c r="D6" s="6"/>
-      <c r="E6" s="4">
-        <v>2</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="6"/>
-    </row>
-    <row r="7" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="4">
-        <v>3</v>
-      </c>
-      <c r="B7" s="5" t="s">
+      <c r="C29" s="17" t="s">
+        <v>40</v>
+      </c>
+      <c r="D29" s="13"/>
+      <c r="E29" s="13"/>
+      <c r="F29" s="14"/>
+      <c r="G29" s="19"/>
+    </row>
+    <row r="30" spans="2:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="22">
         <v>4</v>
       </c>
-      <c r="C7" s="4">
-        <v>1</v>
-      </c>
-      <c r="D7" s="6"/>
-      <c r="E7" s="4">
-        <v>3</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" s="6"/>
-    </row>
-    <row r="8" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="4">
-        <v>4</v>
-      </c>
-      <c r="B8" s="7" t="s">
+      <c r="C30" s="23"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="20"/>
+    </row>
+    <row r="31" spans="2:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="22">
+        <v>5</v>
+      </c>
+      <c r="C31" s="23"/>
+      <c r="D31" s="24"/>
+      <c r="E31" s="24"/>
+      <c r="F31" s="25"/>
+      <c r="G31" s="20"/>
+    </row>
+    <row r="32" spans="2:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="22">
+        <v>6</v>
+      </c>
+      <c r="C32" s="23"/>
+      <c r="D32" s="24"/>
+      <c r="E32" s="24"/>
+      <c r="F32" s="25"/>
+      <c r="G32" s="20"/>
+    </row>
+    <row r="33" spans="2:7" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="22">
+        <v>7</v>
+      </c>
+      <c r="C33" s="23"/>
+      <c r="D33" s="24"/>
+      <c r="E33" s="24"/>
+      <c r="F33" s="25"/>
+      <c r="G33" s="20"/>
+    </row>
+    <row r="34" spans="2:7" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="22">
         <v>8</v>
       </c>
-      <c r="C8" s="4">
-        <v>1</v>
-      </c>
-      <c r="D8" s="6"/>
-      <c r="E8" s="4">
-        <v>4</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" s="6"/>
-    </row>
-    <row r="9" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
-        <v>5</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="4">
-        <v>1</v>
-      </c>
-      <c r="D9" s="6"/>
-      <c r="E9" s="4">
-        <v>5</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="4">
-        <v>6</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" s="4">
-        <v>1</v>
-      </c>
-      <c r="D10" s="6"/>
-      <c r="E10" s="4">
-        <v>6</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" s="6"/>
-    </row>
-    <row r="11" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="4">
-        <v>7</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" s="4">
-        <v>1</v>
-      </c>
-      <c r="D11" s="6"/>
-      <c r="E11" s="4">
-        <v>7</v>
-      </c>
-      <c r="F11" s="8" t="s">
-        <v>23</v>
-      </c>
-      <c r="G11" s="6" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="4">
-        <v>8</v>
-      </c>
-      <c r="B12" s="5" t="s">
+      <c r="C34" s="23"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="20"/>
+    </row>
+    <row r="35" spans="2:7" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="22">
         <v>9</v>
       </c>
-      <c r="C12" s="4">
-        <v>1</v>
-      </c>
-      <c r="D12" s="6"/>
-      <c r="E12" s="4">
-        <v>8</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="G12" s="6"/>
-    </row>
-    <row r="13" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="4">
-        <v>9</v>
-      </c>
-      <c r="B13" s="5" t="s">
+      <c r="C35" s="23"/>
+      <c r="D35" s="24"/>
+      <c r="E35" s="24"/>
+      <c r="F35" s="25"/>
+      <c r="G35" s="20"/>
+    </row>
+    <row r="36" spans="2:7" ht="56.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="26">
         <v>10</v>
       </c>
-      <c r="C13" s="4">
-        <v>1</v>
-      </c>
-      <c r="D13" s="6"/>
-      <c r="E13" s="4">
-        <v>9</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="G13" s="6"/>
-    </row>
-    <row r="14" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="4">
-        <v>10</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C14" s="4">
-        <v>1</v>
-      </c>
-      <c r="D14" s="6"/>
-      <c r="E14" s="4">
-        <v>10</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G14" s="6"/>
-    </row>
-    <row r="15" spans="1:7" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="4">
-        <v>11</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" s="10">
-        <v>1</v>
-      </c>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-    </row>
-    <row r="16" spans="1:7" ht="51" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="4">
-        <v>12</v>
-      </c>
-      <c r="B16" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" s="4">
-        <v>1</v>
-      </c>
-      <c r="D16" s="6"/>
-      <c r="E16" s="6"/>
-      <c r="F16" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="G16" s="6"/>
-    </row>
-    <row r="17" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="4">
-        <v>13</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" s="4">
-        <v>1</v>
-      </c>
-      <c r="D17" s="6"/>
-      <c r="E17" s="6"/>
-      <c r="F17" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="G17" s="6"/>
-    </row>
-    <row r="18" spans="1:7" ht="51" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="4">
-        <v>14</v>
-      </c>
-      <c r="B18" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="C18" s="4">
-        <v>1</v>
-      </c>
-      <c r="D18" s="6"/>
-      <c r="E18" s="6"/>
-      <c r="F18" s="13"/>
-      <c r="G18" s="6"/>
-    </row>
-    <row r="19" spans="1:7" ht="51" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="4">
-        <v>15</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="C19" s="4">
-        <v>1</v>
-      </c>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="6"/>
-    </row>
-    <row r="20" spans="1:7" ht="48.6" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="4">
-        <v>16</v>
-      </c>
-      <c r="B20" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="C20" s="4"/>
-    </row>
+      <c r="C36" s="27"/>
+      <c r="D36" s="28"/>
+      <c r="E36" s="28"/>
+      <c r="F36" s="29"/>
+      <c r="G36" s="21"/>
+    </row>
+    <row r="37" spans="2:7" ht="36" customHeight="1" thickTop="1" x14ac:dyDescent="0.3"/>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A2:G2"/>
+  <mergeCells count="12">
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="B2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
@@ -1147,7 +1510,7 @@
               <x14:cfIcon iconSet="3Symbols2" iconId="2"/>
             </x14:iconSet>
           </x14:cfRule>
-          <xm:sqref>C5:C20</xm:sqref>
+          <xm:sqref>D5:D24</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
           <x14:cfRule type="iconSet" priority="3" id="{17A337BE-4A5D-4888-8CE9-E923E0F43F8C}">
@@ -1166,7 +1529,7 @@
               <x14:cfIcon iconSet="3Symbols2" iconId="2"/>
             </x14:iconSet>
           </x14:cfRule>
-          <xm:sqref>G5:G14</xm:sqref>
+          <xm:sqref>H5:H17</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>

<commit_message>
revisi admin customer tahap 1.3
</commit_message>
<xml_diff>
--- a/DAFTAR REVISI.xlsx
+++ b/DAFTAR REVISI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\V1 Flutter\chupatu_mobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD0E779A-5B62-4528-9F05-7ABA96B3B2A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D397F44-212E-4AB0-8A5D-F6C57188BD16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{408ADA03-67D4-4BA9-9259-15D9795C01CA}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
   <si>
     <t>REVISI CHUPATU MOBILE</t>
   </si>
@@ -157,6 +157,9 @@
   </si>
   <si>
     <t>FITUR CHUPATU PRO INI, NANTI APA MASUK DI LAPORAN PEMASUKAN ATAU GMN YA?</t>
+  </si>
+  <si>
+    <t>sulid</t>
   </si>
 </sst>
 </file>
@@ -1099,7 +1102,9 @@
       <c r="G8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="6"/>
+      <c r="H8" s="6" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="9" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="4">

</xml_diff>

<commit_message>
revisi admin customer tahap 1.5
</commit_message>
<xml_diff>
--- a/DAFTAR REVISI.xlsx
+++ b/DAFTAR REVISI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\V1 Flutter\chupatu_mobile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D397F44-212E-4AB0-8A5D-F6C57188BD16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0ACEBF7-26A3-4C00-82E6-F629A34A6E56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{408ADA03-67D4-4BA9-9259-15D9795C01CA}"/>
+    <workbookView xWindow="5535" yWindow="3510" windowWidth="19575" windowHeight="11295" xr2:uid="{408ADA03-67D4-4BA9-9259-15D9795C01CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="43">
   <si>
     <t>REVISI CHUPATU MOBILE</t>
   </si>
@@ -160,6 +160,9 @@
   </si>
   <si>
     <t>sulid</t>
+  </si>
+  <si>
+    <t>ANTI NAMA DI PROFIL BELUM SINKRON DENGAN HOME UNTUK CUSTOMER, UBAH FOTO PROFIL JUGA GABISA</t>
   </si>
 </sst>
 </file>
@@ -407,7 +410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -431,148 +434,77 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="10">
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -642,6 +574,80 @@
         <scheme val="minor"/>
       </font>
     </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -656,24 +662,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{17F41CE2-7A14-4B5F-8E68-95745F812320}" name="Table4" displayName="Table4" ref="B4:D24" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{17F41CE2-7A14-4B5F-8E68-95745F812320}" name="Table4" displayName="Table4" ref="B4:D24" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
   <autoFilter ref="B4:D24" xr:uid="{17F41CE2-7A14-4B5F-8E68-95745F812320}"/>
   <tableColumns count="3">
-    <tableColumn id="5" xr3:uid="{B811EBC1-E8D7-43F4-AD43-47F971627D50}" name="NO" dataDxfId="0"/>
-    <tableColumn id="2" xr3:uid="{C7960063-BCB1-499F-8687-98DFBC7C5CFF}" name="ADMIN" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{3FCE4E8C-F710-47E1-933B-750F7465C90D}" name="PROGRES" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{B811EBC1-E8D7-43F4-AD43-47F971627D50}" name="NO" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{C7960063-BCB1-499F-8687-98DFBC7C5CFF}" name="ADMIN" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{3FCE4E8C-F710-47E1-933B-750F7465C90D}" name="PROGRES" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D65A9FC3-111E-4033-88B4-1E149CEA158A}" name="Table5" displayName="Table5" ref="F4:H17" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
-  <autoFilter ref="F4:H17" xr:uid="{D65A9FC3-111E-4033-88B4-1E149CEA158A}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{D65A9FC3-111E-4033-88B4-1E149CEA158A}" name="Table5" displayName="Table5" ref="F4:H18" totalsRowShown="0" headerRowDxfId="4" dataDxfId="3">
+  <autoFilter ref="F4:H18" xr:uid="{D65A9FC3-111E-4033-88B4-1E149CEA158A}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{BA4067DE-A9E6-4A79-8183-BBDC9DCB5B98}" name="NO" dataDxfId="7"/>
-    <tableColumn id="2" xr3:uid="{5BEFE63E-C8A9-4CB7-B801-BC4E48F2A3CF}" name="CUSTOMER" dataDxfId="6"/>
-    <tableColumn id="3" xr3:uid="{F876FA39-0709-43F6-9198-5F2408DAB962}" name="PROGRES" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{BA4067DE-A9E6-4A79-8183-BBDC9DCB5B98}" name="NO" dataDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{5BEFE63E-C8A9-4CB7-B801-BC4E48F2A3CF}" name="CUSTOMER" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{F876FA39-0709-43F6-9198-5F2408DAB962}" name="PROGRES" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium14" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -977,30 +983,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01AD129F-D61F-4BD9-AB11-BBB76F78B373}">
   <dimension ref="B2:J37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="9.21875" customWidth="1"/>
-    <col min="3" max="3" width="90.77734375" customWidth="1"/>
-    <col min="4" max="4" width="11.77734375" customWidth="1"/>
-    <col min="5" max="5" width="8.44140625" customWidth="1"/>
-    <col min="6" max="6" width="9.21875" customWidth="1"/>
-    <col min="7" max="7" width="90.77734375" customWidth="1"/>
-    <col min="8" max="8" width="11.77734375" customWidth="1"/>
-    <col min="10" max="10" width="77.21875" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" customWidth="1"/>
+    <col min="3" max="3" width="90.7109375" customWidth="1"/>
+    <col min="4" max="4" width="11.7109375" customWidth="1"/>
+    <col min="5" max="5" width="8.42578125" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" customWidth="1"/>
+    <col min="7" max="7" width="90.7109375" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" customWidth="1"/>
+    <col min="10" max="10" width="77.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:10" ht="23.4" x14ac:dyDescent="0.45">
-      <c r="B2" s="9" t="s">
+    <row r="2" spans="2:10" ht="23.25" x14ac:dyDescent="0.35">
+      <c r="B2" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
-    </row>
-    <row r="4" spans="2:10" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="C2" s="29"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="29"/>
+      <c r="F2" s="29"/>
+      <c r="G2" s="29"/>
+      <c r="H2" s="29"/>
+    </row>
+    <row r="4" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
         <v>25</v>
       </c>
@@ -1021,7 +1027,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="4">
         <v>1</v>
       </c>
@@ -1042,7 +1048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="4">
         <v>2</v>
       </c>
@@ -1063,7 +1069,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="4">
         <v>3</v>
       </c>
@@ -1083,9 +1089,9 @@
       <c r="H7" s="6">
         <v>1</v>
       </c>
-      <c r="J7" s="12"/>
-    </row>
-    <row r="8" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J7" s="9"/>
+    </row>
+    <row r="8" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="4">
         <v>4</v>
       </c>
@@ -1106,7 +1112,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="9" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="4">
         <v>5</v>
       </c>
@@ -1123,9 +1129,11 @@
       <c r="G9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="H9" s="6"/>
-    </row>
-    <row r="10" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H9" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="4">
         <v>6</v>
       </c>
@@ -1142,9 +1150,11 @@
       <c r="G10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H10" s="6"/>
-    </row>
-    <row r="11" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H10" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="4">
         <v>7</v>
       </c>
@@ -1165,7 +1175,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="12" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="4">
         <v>8</v>
       </c>
@@ -1182,9 +1192,11 @@
       <c r="G12" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H12" s="6"/>
-    </row>
-    <row r="13" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H12" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="4">
         <v>9</v>
       </c>
@@ -1201,9 +1213,11 @@
       <c r="G13" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="H13" s="6"/>
-    </row>
-    <row r="14" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H13" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="4">
         <v>10</v>
       </c>
@@ -1220,9 +1234,11 @@
       <c r="G14" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H14" s="6"/>
-    </row>
-    <row r="15" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H14" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="4">
         <v>11</v>
       </c>
@@ -1242,7 +1258,7 @@
       </c>
       <c r="H15" s="6"/>
     </row>
-    <row r="16" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:10" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="4">
         <v>12</v>
       </c>
@@ -1259,9 +1275,11 @@
       <c r="G16" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="H16" s="6"/>
-    </row>
-    <row r="17" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="H16" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="4">
         <v>13</v>
       </c>
@@ -1280,7 +1298,7 @@
       </c>
       <c r="H17" s="6"/>
     </row>
-    <row r="18" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="4">
         <v>14</v>
       </c>
@@ -1291,10 +1309,17 @@
         <v>1</v>
       </c>
       <c r="E18" s="6"/>
-      <c r="F18" s="6"/>
-      <c r="H18" s="6"/>
-    </row>
-    <row r="19" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F18" s="4">
+        <v>14</v>
+      </c>
+      <c r="G18" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="H18" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="51" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="4">
         <v>15</v>
       </c>
@@ -1308,7 +1333,7 @@
       <c r="F19" s="6"/>
       <c r="H19" s="6"/>
     </row>
-    <row r="20" spans="2:8" ht="48.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="2:8" ht="48.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="4">
         <v>16</v>
       </c>
@@ -1317,7 +1342,7 @@
       </c>
       <c r="D20" s="4"/>
     </row>
-    <row r="21" spans="2:8" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="2:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="4">
         <v>17</v>
       </c>
@@ -1326,7 +1351,7 @@
       </c>
       <c r="D21" s="4"/>
     </row>
-    <row r="22" spans="2:8" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="2:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="4">
         <v>18</v>
       </c>
@@ -1335,7 +1360,7 @@
       </c>
       <c r="D22" s="4"/>
     </row>
-    <row r="23" spans="2:8" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="2:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="4">
         <v>19</v>
       </c>
@@ -1344,7 +1369,7 @@
       </c>
       <c r="D23" s="4"/>
     </row>
-    <row r="24" spans="2:8" ht="46.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="2:8" ht="46.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B24" s="4">
         <v>20</v>
       </c>
@@ -1353,129 +1378,127 @@
       </c>
       <c r="D24" s="4"/>
     </row>
-    <row r="25" spans="2:8" ht="46.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="26" spans="2:8" ht="46.2" customHeight="1" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="15" t="s">
+    <row r="25" spans="2:8" ht="46.15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="26" spans="2:8" ht="46.15" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C26" s="16" t="s">
+      <c r="C26" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="11"/>
-      <c r="G26" s="18"/>
-    </row>
-    <row r="27" spans="2:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="22">
-        <v>1</v>
-      </c>
-      <c r="C27" s="17" t="s">
+      <c r="D26" s="21"/>
+      <c r="E26" s="21"/>
+      <c r="F26" s="22"/>
+      <c r="G26" s="12"/>
+    </row>
+    <row r="27" spans="2:8" ht="56.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="15">
+        <v>1</v>
+      </c>
+      <c r="C27" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="D27" s="13"/>
-      <c r="E27" s="13"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="19"/>
-    </row>
-    <row r="28" spans="2:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="22">
+      <c r="D27" s="24"/>
+      <c r="E27" s="24"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="10"/>
+    </row>
+    <row r="28" spans="2:8" ht="56.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B28" s="15">
         <v>2</v>
       </c>
-      <c r="C28" s="17" t="str">
-        <f>UPPER("anti nama di profil belum sinkron dengan home untuk customer, ubah foto profil juga gabisa")</f>
-        <v>ANTI NAMA DI PROFIL BELUM SINKRON DENGAN HOME UNTUK CUSTOMER, UBAH FOTO PROFIL JUGA GABISA</v>
-      </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="13"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="19"/>
-    </row>
-    <row r="29" spans="2:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="22">
+      <c r="C28" s="23" t="s">
+        <v>40</v>
+      </c>
+      <c r="D28" s="30"/>
+      <c r="E28" s="30"/>
+      <c r="F28" s="25"/>
+      <c r="G28" s="10"/>
+    </row>
+    <row r="29" spans="2:8" ht="56.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="15">
         <v>3</v>
       </c>
-      <c r="C29" s="17" t="s">
-        <v>40</v>
-      </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="13"/>
-      <c r="F29" s="14"/>
-      <c r="G29" s="19"/>
-    </row>
-    <row r="30" spans="2:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="22">
+      <c r="C29" s="23"/>
+      <c r="D29" s="24"/>
+      <c r="E29" s="24"/>
+      <c r="F29" s="25"/>
+      <c r="G29" s="10"/>
+    </row>
+    <row r="30" spans="2:8" ht="56.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B30" s="15">
         <v>4</v>
       </c>
-      <c r="C30" s="23"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="24"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="20"/>
-    </row>
-    <row r="31" spans="2:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="22">
+      <c r="C30" s="26"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
+      <c r="F30" s="28"/>
+      <c r="G30" s="13"/>
+    </row>
+    <row r="31" spans="2:8" ht="56.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="15">
         <v>5</v>
       </c>
-      <c r="C31" s="23"/>
-      <c r="D31" s="24"/>
-      <c r="E31" s="24"/>
-      <c r="F31" s="25"/>
-      <c r="G31" s="20"/>
-    </row>
-    <row r="32" spans="2:8" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="22">
+      <c r="C31" s="26"/>
+      <c r="D31" s="27"/>
+      <c r="E31" s="27"/>
+      <c r="F31" s="28"/>
+      <c r="G31" s="13"/>
+    </row>
+    <row r="32" spans="2:8" ht="56.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="15">
         <v>6</v>
       </c>
-      <c r="C32" s="23"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="24"/>
-      <c r="F32" s="25"/>
-      <c r="G32" s="20"/>
-    </row>
-    <row r="33" spans="2:7" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="22">
+      <c r="C32" s="26"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="28"/>
+      <c r="G32" s="13"/>
+    </row>
+    <row r="33" spans="2:7" ht="56.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B33" s="15">
         <v>7</v>
       </c>
-      <c r="C33" s="23"/>
-      <c r="D33" s="24"/>
-      <c r="E33" s="24"/>
-      <c r="F33" s="25"/>
-      <c r="G33" s="20"/>
-    </row>
-    <row r="34" spans="2:7" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="22">
+      <c r="C33" s="26"/>
+      <c r="D33" s="27"/>
+      <c r="E33" s="27"/>
+      <c r="F33" s="28"/>
+      <c r="G33" s="13"/>
+    </row>
+    <row r="34" spans="2:7" ht="56.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B34" s="15">
         <v>8</v>
       </c>
-      <c r="C34" s="23"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="24"/>
-      <c r="F34" s="25"/>
-      <c r="G34" s="20"/>
-    </row>
-    <row r="35" spans="2:7" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="22">
+      <c r="C34" s="26"/>
+      <c r="D34" s="27"/>
+      <c r="E34" s="27"/>
+      <c r="F34" s="28"/>
+      <c r="G34" s="13"/>
+    </row>
+    <row r="35" spans="2:7" ht="56.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B35" s="15">
         <v>9</v>
       </c>
-      <c r="C35" s="23"/>
-      <c r="D35" s="24"/>
-      <c r="E35" s="24"/>
-      <c r="F35" s="25"/>
-      <c r="G35" s="20"/>
-    </row>
-    <row r="36" spans="2:7" ht="56.4" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B36" s="26">
+      <c r="C35" s="26"/>
+      <c r="D35" s="27"/>
+      <c r="E35" s="27"/>
+      <c r="F35" s="28"/>
+      <c r="G35" s="13"/>
+    </row>
+    <row r="36" spans="2:7" ht="56.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="16">
         <v>10</v>
       </c>
-      <c r="C36" s="27"/>
-      <c r="D36" s="28"/>
-      <c r="E36" s="28"/>
-      <c r="F36" s="29"/>
-      <c r="G36" s="21"/>
-    </row>
-    <row r="37" spans="2:7" ht="36" customHeight="1" thickTop="1" x14ac:dyDescent="0.3"/>
+      <c r="C36" s="17"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="19"/>
+      <c r="G36" s="14"/>
+    </row>
+    <row r="37" spans="2:7" ht="36" customHeight="1" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="B2:H2"/>
     <mergeCell ref="C36:F36"/>
     <mergeCell ref="C26:F26"/>
     <mergeCell ref="C27:F27"/>
@@ -1487,7 +1510,6 @@
     <mergeCell ref="C33:F33"/>
     <mergeCell ref="C34:F34"/>
     <mergeCell ref="C35:F35"/>
-    <mergeCell ref="B2:H2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" r:id="rId1"/>
@@ -1534,7 +1556,7 @@
               <x14:cfIcon iconSet="3Symbols2" iconId="2"/>
             </x14:iconSet>
           </x14:cfRule>
-          <xm:sqref>H5:H17</xm:sqref>
+          <xm:sqref>H5:H18</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>